<commit_message>
Results: Live 100-user 60s baseline load test (230,739 reqs, 3811 RPS, 14.58ms avg) & updated Excel report
</commit_message>
<xml_diff>
--- a/automated_test/BlockCertify_2.0_E2E_Security_Load_Report.xlsx
+++ b/automated_test/BlockCertify_2.0_E2E_Security_Load_Report.xlsx
@@ -698,7 +698,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>GitHub: github.com/dhanushvk18/Blockcertify2.0  |  Generated: 05 Aug 2026 13:27</t>
+          <t>GitHub: github.com/dhanushvk18/Blockcertify2.0  |  Generated: 05 Aug 2026 13:59</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>2054.84</v>
+        <v>3811.32</v>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>36.91 ms</t>
+          <t>14.58 ms</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>1.11 ms</t>
+          <t>0.28 ms</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>7806.8 ms</t>
+          <t>2325.06 ms</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>123390</v>
+        <v>230739</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>60</v>
+        <v>60.54</v>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>123390</v>
+        <v>230739</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>2054.84</v>
+        <v>3811.32</v>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
@@ -1334,7 +1334,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>36.91</v>
+        <v>14.58</v>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>1.11</v>
+        <v>0.28</v>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>7806.8</v>
+        <v>2325.06</v>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>

</xml_diff>